<commit_message>
Add formula rows (合计/税金合计/股利利息合计) + tax-rate columns + warning to 表外数据收集表
</commit_message>
<xml_diff>
--- a/examples/表外数据收集表.xlsx
+++ b/examples/表外数据收集表.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表外数据收集表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="表外数据收集表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="8">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00;-#,##0.00;-"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,11 +34,23 @@
     </font>
     <font>
       <name val="宋体"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="宋体"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
       <sz val="11"/>
     </font>
     <font>
@@ -47,21 +61,21 @@
     <font>
       <name val="宋体"/>
       <b val="1"/>
-      <color rgb="00006100"/>
-      <sz val="10"/>
+      <color rgb="009C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="宋体"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="00C00000"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -70,7 +84,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -85,7 +114,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,7 +128,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -108,38 +142,79 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -506,13 +581,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -522,829 +599,1001 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>编制现金流量表所需表外数据 —— 在白色'金额'栏填写，其余列不要改动</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>⚠ 重要提醒：粉红阴影部分已设置为公式，数据自动计算产生，务请不要填入任何数据以免出错！只需在「金额」栏白色空格内录入数据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>一、编制现金流量表所需数据录入</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>项  目</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>金  额</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>税  率</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>税率说明</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>说  明</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>应收票据贴现利息支出</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>票据贴现产生的利息（如无贴现可留空）</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+    <row r="6">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>支付给职工的工资</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>全年实发工资总额（含奖金津贴）★直接影响经营净额</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>全年实发工资总额（含奖金津贴）★必填，直接影响经营净额</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>支付给职工的四金</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>800000</v>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>社保+公积金等（不填则按工资×26.6%自动推算）</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+    <row r="8">
+      <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>支付给职工的其他福利费</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>其他职工福利（不填则按工资×1.06%自动推算）</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+    <row r="9">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="C9" s="14">
+        <f>C8+C7+C6</f>
+        <v/>
+      </c>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>(公式：工资+四金+福利费)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>销项税额</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="16" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>须根据实际税率修改</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>全年销项税额（不填则按收入×6%推算，请按实际税率改）</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>进项税额</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>须根据实际税率修改</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>全年进项税额（不填则按成本×6%推算）</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
+    <row r="12">
+      <c r="A12" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>应交增值税</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>销项−进项（不填自动计算）</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>销项−进项（不填则由引擎自动按销项-进项算）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>其他各项税</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>除增值税外各税种（不填取利润表营业税金及附加）</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
+    <row r="14">
+      <c r="A14" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>所得税</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>须根据实际税率修改</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>全年所得税（不填取利润表所得税费用）</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>管理费用中列支的税金</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>计入管理费用的税金（如房产税、印花税）</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
+    <row r="16">
+      <c r="A16" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>在其他业务支出中列支的税金</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="9" t="inlineStr"/>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>其他业务负担的税金</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
+    <row r="17">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>实际应缴纳各项税金合计</t>
+        </is>
+      </c>
+      <c r="C17" s="14">
+        <f>C16+C15+C14+C13+C12</f>
+        <v/>
+      </c>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>(公式：其他业务税金+管理税金+所得税+其他各项税+应交增值税)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>分配股利所支付的现金</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="9" t="inlineStr"/>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>全年向股东分配股利支付的现金</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
+    <row r="19">
+      <c r="A19" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>分配利润所支付的现金</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="9" t="inlineStr"/>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>全年分配利润支付的现金</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
+    <row r="20">
+      <c r="A20" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>利息支出</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="9" t="inlineStr"/>
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>利息支出总额（不抵减利息收入；即利润表财务费用中的利息部分）</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
+    <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>分配股利、利润或偿付利息所支付的现金</t>
+        </is>
+      </c>
+      <c r="C21" s="14">
+        <f>C20+C19+C18</f>
+        <v/>
+      </c>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>(公式：利息支出+分配利润+分配股利)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>计提坏账准备的比率</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="16" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>可根据实际计提比率修改</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>坏账计提比例（默认0.5%，按公司实际改）</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
+    <row r="23">
+      <c r="A23" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>计提的坏账准备</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="9" t="inlineStr"/>
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>当年计提坏账（不填为0，与模板口径一致）</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
+    <row r="24">
+      <c r="A24" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>无形资产摊销</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="9" t="inlineStr"/>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>当年无形资产摊销额</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
+    <row r="25">
+      <c r="A25" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>长期待摊费用摊销</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="9" t="inlineStr"/>
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>当年长期待摊费用摊销额</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
+    <row r="26">
+      <c r="A26" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>固定资产报废损失</t>
         </is>
       </c>
-      <c r="C22" s="13" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="9" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>当年报废损失（不计入处置现金净额）</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
+    <row r="27">
+      <c r="A27" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>收到投资分红或利润</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="9" t="inlineStr"/>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>当年收到的对外投资分红/利润</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
+    <row r="28">
+      <c r="A28" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>处置固定资产收回的现金净额</t>
         </is>
       </c>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="9" t="inlineStr"/>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>处置固定资产收到的现金净额</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
+    <row r="29">
+      <c r="A29" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>处置无形资产收回的现金净额</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="9" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>处置无形资产收到的现金净额</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
+    <row r="30">
+      <c r="A30" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>处置其他长期资产收回的现金净额</t>
         </is>
       </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="9" t="inlineStr"/>
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>处置其他长期资产收到的现金净额</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
+    <row r="31">
+      <c r="A31" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>收到的其他与投资活动有关的现金</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="9" t="inlineStr"/>
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>投资活动其他现金流入</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
+    <row r="32">
+      <c r="A32" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>支付的其他与投资活动有关的现金</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="9" t="inlineStr"/>
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>投资活动其他现金流出</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
+    <row r="33">
+      <c r="A33" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>收到的其他与筹资活动有关的现金</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="9" t="inlineStr"/>
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>筹资活动其他现金流入</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
+    <row r="34">
+      <c r="A34" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>偿还债务所支付的现金</t>
         </is>
       </c>
-      <c r="C30" s="13" t="n">
-        <v>9000000</v>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="9" t="inlineStr"/>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>偿还债务本金支付的现金（不填则按借款变动自动倒挤）</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
+    <row r="35">
+      <c r="A35" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>支付的其他与筹资活动有关的现金</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="9" t="inlineStr"/>
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>筹资活动其他现金流出</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
+    <row r="36">
+      <c r="A36" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>汇率变动对现金的影响</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="9" t="inlineStr"/>
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>外币折算对现金的影响（无外币业务填0）</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
+    <row r="37">
+      <c r="A37" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>现金等价物期末余额</t>
         </is>
       </c>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="9" t="inlineStr"/>
+      <c r="F37" s="9" t="inlineStr">
         <is>
           <t>如有现金等价物（一般企业可留空）</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
+    <row r="38">
+      <c r="A38" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>现金等价物期初余额</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="9" t="inlineStr"/>
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>如有现金等价物（一般企业可留空）</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
+    <row r="39">
+      <c r="A39" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>支付的其他与经营活动有关的现金</t>
         </is>
       </c>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="9" t="inlineStr"/>
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>经营活动其他现金流出（不填则由平衡项自动倒挤）</t>
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>【高精度模式·可选】以下从现金流量表主表直接抄真实值，填了即用真实值替代公式推算，误差可压到 ±1% 以内</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>二、【高精度模式·可选】从现金流量表主表直接抄真实值</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B42" s="18" t="inlineStr">
         <is>
           <t>项  目</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
+      <c r="C42" s="18" t="inlineStr">
         <is>
           <t>金  额</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="D42" s="18" t="inlineStr"/>
+      <c r="E42" s="19" t="n"/>
+      <c r="F42" s="18" t="inlineStr">
+        <is>
+          <t>说  明</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>销售商品提供劳务收到的现金</t>
         </is>
       </c>
-      <c r="C39" s="13" t="n">
-        <v>60550000</v>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"销售商品、提供劳务收到的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
+    <row r="44">
+      <c r="A44" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>收到的税费返还</t>
         </is>
       </c>
-      <c r="C40" s="13" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="C44" s="7" t="n"/>
+      <c r="D44" s="20" t="n"/>
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"收到的税费返还"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
+    <row r="45">
+      <c r="A45" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>购买商品接受劳务支付的现金</t>
         </is>
       </c>
-      <c r="C41" s="13" t="n">
-        <v>42500000</v>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="C45" s="7" t="n"/>
+      <c r="D45" s="20" t="n"/>
+      <c r="F45" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"购买商品、接受劳务支付的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
+    <row r="46">
+      <c r="A46" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>支付给职工以及为职工支付的现金</t>
         </is>
       </c>
-      <c r="C42" s="13" t="n">
-        <v>6800000</v>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="C46" s="7" t="n"/>
+      <c r="D46" s="20" t="n"/>
+      <c r="F46" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"支付给职工以及为职工支付的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="n">
+    <row r="47">
+      <c r="A47" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>支付的各项税费</t>
         </is>
       </c>
-      <c r="C43" s="13" t="n">
-        <v>2300000</v>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="20" t="n"/>
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"支付的各项税费"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
+    <row r="48">
+      <c r="A48" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>收到的其他与经营活动有关的现金</t>
         </is>
       </c>
-      <c r="C44" s="13" t="n">
-        <v>500000</v>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="20" t="n"/>
+      <c r="F48" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"收到的其他与经营活动有关的现金"（高精度模式，选填）★填此项后经营净额不再倒挤，按各项真实值求和</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
+    <row r="49">
+      <c r="A49" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>支付的其他与经营活动有关的现金</t>
         </is>
       </c>
-      <c r="C45" s="13" t="n">
-        <v>3100000</v>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="20" t="n"/>
+      <c r="F49" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"支付的其他与经营活动有关的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
+    <row r="50">
+      <c r="A50" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>购建固定资产无形资产和其他长期资产支付的现金</t>
         </is>
       </c>
-      <c r="C46" s="13" t="n">
-        <v>3100000</v>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>现金流量表主表"购建固定资产、无形资产和其他长期资产支付的现金"（高精度模式，选填）</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="20" t="n"/>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>现金流量表主表"购建固定资产、无形资产和其他长期资产所支付的现金"（高精度模式，选填）</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>投资所支付的现金</t>
         </is>
       </c>
-      <c r="C47" s="13" t="n">
-        <v>500000</v>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="20" t="n"/>
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"投资所支付的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
+    <row r="52">
+      <c r="A52" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>吸收投资所收到的现金</t>
         </is>
       </c>
-      <c r="C48" s="6" t="n"/>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="C52" s="7" t="n"/>
+      <c r="D52" s="20" t="n"/>
+      <c r="F52" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"吸收投资收到的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
+    <row r="53">
+      <c r="A53" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>借款所收到的现金</t>
         </is>
       </c>
-      <c r="C49" s="13" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="C53" s="7" t="n"/>
+      <c r="D53" s="20" t="n"/>
+      <c r="F53" s="9" t="inlineStr">
         <is>
           <t>现金流量表主表"借款收到的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="21" t="inlineStr">
         <is>
           <t>※ ★ 必填项只有：支付给职工的工资。其余均可留空由引擎自动推算/置0。</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="12" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="21" t="inlineStr">
         <is>
           <t>※ ★ 金额单位：元。直接填数字，不要带千分位逗号。</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="21" t="inlineStr">
+        <is>
+          <t>※ ★ 粉红阴影 = 公式自动算，不要手填（手填会让 Excel 报错）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="21" t="inlineStr">
+        <is>
+          <t>※ ★ 税率列默认值与原模板一致（销项 6% / 进项 0% / 所得税 25% / 坏账 0.5%），请按公司实际修改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="21" t="inlineStr">
         <is>
           <t>※ ★ 填完后保存，运行时作为 --extra 参数传入：python cash_flow_generator.py --bs 资产负债表 --pl 利润表 --extra 表外数据收集表.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="12" t="inlineStr">
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="21" t="inlineStr">
         <is>
           <t>※ ★ 补齐本表后，'经营活动产生的现金流量净额'精度可由 ±20% 提升至 ±5% 以内。</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="12" t="inlineStr">
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="21" t="inlineStr">
         <is>
           <t>※ ★ 数据来源建议：工资表/社保申报表、增值税及所得税申报表、固定资产折旧明细表、银行对账单。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A51:D51"/>
+  <mergeCells count="23">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 应交增值税 formula row (pink, =销项-进项); broaden {rk} to reference any above row
</commit_message>
<xml_diff>
--- a/examples/表外数据收集表.xlsx
+++ b/examples/表外数据收集表.xlsx
@@ -785,26 +785,27 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>应交增值税</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>销项−进项（不填则由引擎自动按销项-进项算）</t>
+      <c r="C12" s="14">
+        <f>C10-C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>(公式：销项税额-进项税额)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
@@ -822,7 +823,7 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
@@ -846,7 +847,7 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
@@ -864,7 +865,7 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
@@ -901,7 +902,7 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
@@ -919,7 +920,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
@@ -937,7 +938,7 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
@@ -974,7 +975,7 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
@@ -998,7 +999,7 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
@@ -1016,7 +1017,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
@@ -1034,7 +1035,7 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
@@ -1052,7 +1053,7 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
@@ -1070,7 +1071,7 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
@@ -1088,7 +1089,7 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
@@ -1106,7 +1107,7 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
@@ -1124,7 +1125,7 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
@@ -1142,7 +1143,7 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
@@ -1160,7 +1161,7 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
@@ -1178,7 +1179,7 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
@@ -1196,7 +1197,7 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
@@ -1214,7 +1215,7 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
@@ -1232,7 +1233,7 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
@@ -1250,7 +1251,7 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
@@ -1268,7 +1269,7 @@
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
@@ -1286,7 +1287,7 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 数据来源 column (浅蓝) for audit trail of manual data entries
</commit_message>
<xml_diff>
--- a/examples/表外数据收集表.xlsx
+++ b/examples/表外数据收集表.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00;-#,##0.00;-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,12 @@
     </font>
     <font>
       <name val="宋体"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="宋体"/>
       <b val="1"/>
       <color rgb="009C0006"/>
       <sz val="11"/>
@@ -75,7 +81,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +111,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -167,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -192,28 +203,39 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="10" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -581,15 +603,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -599,10 +622,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>⚠ 重要提醒：粉红阴影部分已设置为公式，数据自动计算产生，务请不要填入任何数据以免出错！只需在「金额」栏白色空格内录入数据。</t>
+          <t>⚠ 重要提醒：粉红阴影部分已设置为公式，数据自动计算产生，务请不要填入任何数据以免出错！只需在「金额」栏白色空格内录入数据。建议在「数据来源」栏填写每个数字的出处（如'管理费用明细表-工资'），方便审计追溯。</t>
         </is>
       </c>
     </row>
@@ -640,6 +663,11 @@
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>数据来源</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>说  明</t>
         </is>
@@ -657,7 +685,8 @@
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="8" t="n"/>
       <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>票据贴现产生的利息（如无贴现可留空）</t>
         </is>
@@ -667,15 +696,16 @@
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>支付给职工的工资</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n"/>
+      <c r="C6" s="13" t="n"/>
       <c r="D6" s="8" t="n"/>
       <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>全年实发工资总额（含奖金津贴）★必填，直接影响经营净额</t>
         </is>
@@ -693,7 +723,8 @@
       <c r="C7" s="7" t="n"/>
       <c r="D7" s="8" t="n"/>
       <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>社保+公积金等（不填则按工资×26.6%自动推算）</t>
         </is>
@@ -711,26 +742,28 @@
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>其他职工福利（不填则按工资×1.06%自动推算）</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="n"/>
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="16">
         <f>C8+C7+C6</f>
         <v/>
       </c>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="14" t="n"/>
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>(公式：工资+四金+福利费)</t>
         </is>
@@ -746,7 +779,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n"/>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.06</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -754,7 +787,8 @@
           <t>须根据实际税率修改</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>全年销项税额（不填则按收入×6%推算，请按实际税率改）</t>
         </is>
@@ -770,7 +804,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n"/>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -778,26 +812,28 @@
           <t>须根据实际税率修改</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>全年进项税额（不填则按成本×6%推算）</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="n"/>
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>应交增值税</t>
         </is>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="16">
         <f>C10-C11</f>
         <v/>
       </c>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="15" t="inlineStr">
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>(公式：销项税额-进项税额)</t>
         </is>
@@ -815,7 +851,8 @@
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="8" t="n"/>
       <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>除增值税外各税种（不填取利润表营业税金及附加）</t>
         </is>
@@ -831,7 +868,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="n"/>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="18" t="n">
         <v>0.25</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -839,7 +876,8 @@
           <t>须根据实际税率修改</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>全年所得税（不填取利润表所得税费用）</t>
         </is>
@@ -857,7 +895,8 @@
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="9" t="inlineStr"/>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>计入管理费用的税金（如房产税、印花税）</t>
         </is>
@@ -875,26 +914,28 @@
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="9" t="inlineStr"/>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>其他业务负担的税金</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="n"/>
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>实际应缴纳各项税金合计</t>
         </is>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="16">
         <f>C16+C15+C14+C13+C12</f>
         <v/>
       </c>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>(公式：其他业务税金+管理税金+所得税+其他各项税+应交增值税)</t>
         </is>
@@ -912,7 +953,8 @@
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="9" t="inlineStr"/>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>全年向股东分配股利支付的现金</t>
         </is>
@@ -930,7 +972,8 @@
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="8" t="n"/>
       <c r="E19" s="9" t="inlineStr"/>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>全年分配利润支付的现金</t>
         </is>
@@ -948,26 +991,28 @@
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="9" t="inlineStr"/>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>利息支出总额（不抵减利息收入；即利润表财务费用中的利息部分）</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n"/>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="A21" s="14" t="n"/>
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>分配股利、利润或偿付利息所支付的现金</t>
         </is>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="16">
         <f>C20+C19+C18</f>
         <v/>
       </c>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>(公式：利息支出+分配利润+分配股利)</t>
         </is>
@@ -983,7 +1028,7 @@
         </is>
       </c>
       <c r="C22" s="7" t="n"/>
-      <c r="D22" s="16" t="n">
+      <c r="D22" s="18" t="n">
         <v>0.005</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -991,7 +1036,8 @@
           <t>可根据实际计提比率修改</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>坏账计提比例（默认0.5%，按公司实际改）</t>
         </is>
@@ -1009,7 +1055,8 @@
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="9" t="inlineStr"/>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>当年计提坏账（不填为0，与模板口径一致）</t>
         </is>
@@ -1027,7 +1074,8 @@
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="9" t="inlineStr"/>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>当年无形资产摊销额</t>
         </is>
@@ -1045,7 +1093,8 @@
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="9" t="inlineStr"/>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>当年长期待摊费用摊销额</t>
         </is>
@@ -1063,7 +1112,8 @@
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="8" t="n"/>
       <c r="E26" s="9" t="inlineStr"/>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>当年报废损失（不计入处置现金净额）</t>
         </is>
@@ -1081,7 +1131,8 @@
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="8" t="n"/>
       <c r="E27" s="9" t="inlineStr"/>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>当年收到的对外投资分红/利润</t>
         </is>
@@ -1099,7 +1150,8 @@
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="8" t="n"/>
       <c r="E28" s="9" t="inlineStr"/>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="11" t="inlineStr">
         <is>
           <t>处置固定资产收到的现金净额</t>
         </is>
@@ -1117,7 +1169,8 @@
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="9" t="inlineStr"/>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>处置无形资产收到的现金净额</t>
         </is>
@@ -1135,7 +1188,8 @@
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="9" t="inlineStr"/>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>处置其他长期资产收到的现金净额</t>
         </is>
@@ -1153,7 +1207,8 @@
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="8" t="n"/>
       <c r="E31" s="9" t="inlineStr"/>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>投资活动其他现金流入</t>
         </is>
@@ -1171,7 +1226,8 @@
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="8" t="n"/>
       <c r="E32" s="9" t="inlineStr"/>
-      <c r="F32" s="9" t="inlineStr">
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="11" t="inlineStr">
         <is>
           <t>投资活动其他现金流出</t>
         </is>
@@ -1189,7 +1245,8 @@
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="8" t="n"/>
       <c r="E33" s="9" t="inlineStr"/>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>筹资活动其他现金流入</t>
         </is>
@@ -1207,7 +1264,8 @@
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="8" t="n"/>
       <c r="E34" s="9" t="inlineStr"/>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="11" t="inlineStr">
         <is>
           <t>偿还债务本金支付的现金（不填则按借款变动自动倒挤）</t>
         </is>
@@ -1225,7 +1283,8 @@
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="8" t="n"/>
       <c r="E35" s="9" t="inlineStr"/>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>筹资活动其他现金流出</t>
         </is>
@@ -1243,7 +1302,8 @@
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="8" t="n"/>
       <c r="E36" s="9" t="inlineStr"/>
-      <c r="F36" s="9" t="inlineStr">
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>外币折算对现金的影响（无外币业务填0）</t>
         </is>
@@ -1261,7 +1321,8 @@
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="8" t="n"/>
       <c r="E37" s="9" t="inlineStr"/>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>如有现金等价物（一般企业可留空）</t>
         </is>
@@ -1279,7 +1340,8 @@
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="8" t="n"/>
       <c r="E38" s="9" t="inlineStr"/>
-      <c r="F38" s="9" t="inlineStr">
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="11" t="inlineStr">
         <is>
           <t>如有现金等价物（一般企业可留空）</t>
         </is>
@@ -1297,38 +1359,44 @@
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="8" t="n"/>
       <c r="E39" s="9" t="inlineStr"/>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="F39" s="10" t="n"/>
+      <c r="G39" s="11" t="inlineStr">
         <is>
           <t>经营活动其他现金流出（不填则由平衡项自动倒挤）</t>
         </is>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>二、【高精度模式·可选】从现金流量表主表直接抄真实值</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="18" t="inlineStr">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B42" s="18" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>项  目</t>
         </is>
       </c>
-      <c r="C42" s="18" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
         <is>
           <t>金  额</t>
         </is>
       </c>
-      <c r="D42" s="18" t="inlineStr"/>
-      <c r="E42" s="19" t="n"/>
-      <c r="F42" s="18" t="inlineStr">
+      <c r="D42" s="20" t="inlineStr"/>
+      <c r="E42" s="21" t="n"/>
+      <c r="F42" s="20" t="inlineStr">
+        <is>
+          <t>数据来源</t>
+        </is>
+      </c>
+      <c r="G42" s="20" t="inlineStr">
         <is>
           <t>说  明</t>
         </is>
@@ -1344,8 +1412,9 @@
         </is>
       </c>
       <c r="C43" s="7" t="n"/>
-      <c r="D43" s="20" t="n"/>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="D43" s="22" t="n"/>
+      <c r="F43" s="23" t="n"/>
+      <c r="G43" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"销售商品、提供劳务收到的现金"（高精度模式，选填）</t>
         </is>
@@ -1361,8 +1430,9 @@
         </is>
       </c>
       <c r="C44" s="7" t="n"/>
-      <c r="D44" s="20" t="n"/>
-      <c r="F44" s="9" t="inlineStr">
+      <c r="D44" s="22" t="n"/>
+      <c r="F44" s="23" t="n"/>
+      <c r="G44" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"收到的税费返还"（高精度模式，选填）</t>
         </is>
@@ -1378,8 +1448,9 @@
         </is>
       </c>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="20" t="n"/>
-      <c r="F45" s="9" t="inlineStr">
+      <c r="D45" s="22" t="n"/>
+      <c r="F45" s="23" t="n"/>
+      <c r="G45" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"购买商品、接受劳务支付的现金"（高精度模式，选填）</t>
         </is>
@@ -1395,8 +1466,9 @@
         </is>
       </c>
       <c r="C46" s="7" t="n"/>
-      <c r="D46" s="20" t="n"/>
-      <c r="F46" s="9" t="inlineStr">
+      <c r="D46" s="22" t="n"/>
+      <c r="F46" s="23" t="n"/>
+      <c r="G46" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"支付给职工以及为职工支付的现金"（高精度模式，选填）</t>
         </is>
@@ -1412,8 +1484,9 @@
         </is>
       </c>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="20" t="n"/>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="D47" s="22" t="n"/>
+      <c r="F47" s="23" t="n"/>
+      <c r="G47" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"支付的各项税费"（高精度模式，选填）</t>
         </is>
@@ -1429,8 +1502,9 @@
         </is>
       </c>
       <c r="C48" s="7" t="n"/>
-      <c r="D48" s="20" t="n"/>
-      <c r="F48" s="9" t="inlineStr">
+      <c r="D48" s="22" t="n"/>
+      <c r="F48" s="23" t="n"/>
+      <c r="G48" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"收到的其他与经营活动有关的现金"（高精度模式，选填）★填此项后经营净额不再倒挤，按各项真实值求和</t>
         </is>
@@ -1446,8 +1520,9 @@
         </is>
       </c>
       <c r="C49" s="7" t="n"/>
-      <c r="D49" s="20" t="n"/>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="D49" s="22" t="n"/>
+      <c r="F49" s="23" t="n"/>
+      <c r="G49" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"支付的其他与经营活动有关的现金"（高精度模式，选填）</t>
         </is>
@@ -1463,8 +1538,9 @@
         </is>
       </c>
       <c r="C50" s="7" t="n"/>
-      <c r="D50" s="20" t="n"/>
-      <c r="F50" s="9" t="inlineStr">
+      <c r="D50" s="22" t="n"/>
+      <c r="F50" s="23" t="n"/>
+      <c r="G50" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"购建固定资产、无形资产和其他长期资产所支付的现金"（高精度模式，选填）</t>
         </is>
@@ -1480,8 +1556,9 @@
         </is>
       </c>
       <c r="C51" s="7" t="n"/>
-      <c r="D51" s="20" t="n"/>
-      <c r="F51" s="9" t="inlineStr">
+      <c r="D51" s="22" t="n"/>
+      <c r="F51" s="23" t="n"/>
+      <c r="G51" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"投资所支付的现金"（高精度模式，选填）</t>
         </is>
@@ -1497,8 +1574,9 @@
         </is>
       </c>
       <c r="C52" s="7" t="n"/>
-      <c r="D52" s="20" t="n"/>
-      <c r="F52" s="9" t="inlineStr">
+      <c r="D52" s="22" t="n"/>
+      <c r="F52" s="23" t="n"/>
+      <c r="G52" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"吸收投资收到的现金"（高精度模式，选填）</t>
         </is>
@@ -1514,86 +1592,95 @@
         </is>
       </c>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="20" t="n"/>
-      <c r="F53" s="9" t="inlineStr">
+      <c r="D53" s="22" t="n"/>
+      <c r="F53" s="23" t="n"/>
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>现金流量表主表"借款收到的现金"（高精度模式，选填）</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="21" t="inlineStr">
+      <c r="A55" s="24" t="inlineStr">
         <is>
           <t>※ ★ 必填项只有：支付给职工的工资。其余均可留空由引擎自动推算/置0。</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="21" t="inlineStr">
+      <c r="A56" s="24" t="inlineStr">
         <is>
           <t>※ ★ 金额单位：元。直接填数字，不要带千分位逗号。</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="21" t="inlineStr">
+      <c r="A57" s="24" t="inlineStr">
         <is>
           <t>※ ★ 粉红阴影 = 公式自动算，不要手填（手填会让 Excel 报错）。</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="21" t="inlineStr">
+      <c r="A58" s="24" t="inlineStr">
         <is>
           <t>※ ★ 税率列默认值与原模板一致（销项 6% / 进项 0% / 所得税 25% / 坏账 0.5%），请按公司实际修改。</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="21" t="inlineStr">
+      <c r="A59" s="24" t="inlineStr">
+        <is>
+          <t>※ ★ 数据来源列（浅蓝）：建议每填一个数字就在这列注明出处（如'管理费用明细-工资'、'税务申报表-增值税'），便于审计追溯。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="24" t="inlineStr">
         <is>
           <t>※ ★ 填完后保存，运行时作为 --extra 参数传入：python cash_flow_generator.py --bs 资产负债表 --pl 利润表 --extra 表外数据收集表.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="21" t="inlineStr">
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="24" t="inlineStr">
         <is>
           <t>※ ★ 补齐本表后，'经营活动产生的现金流量净额'精度可由 ±20% 提升至 ±5% 以内。</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="21" t="inlineStr">
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="24" t="inlineStr">
         <is>
           <t>※ ★ 数据来源建议：工资表/社保申报表、增值税及所得税申报表、固定资产折旧明细表、银行对账单。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A41:F41"/>
+  <mergeCells count="24">
+    <mergeCell ref="A62:G62"/>
     <mergeCell ref="D46:E46"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="D50:E50"/>
     <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A57:F57"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="D52:E52"/>
     <mergeCell ref="D49:E49"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A60:G60"/>
     <mergeCell ref="D48:E48"/>
     <mergeCell ref="D53:E53"/>
     <mergeCell ref="D47:E47"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A41:G41"/>
     <mergeCell ref="D42:E42"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A56:G56"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A55:G55"/>
     <mergeCell ref="D51:E51"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A57:G57"/>
     <mergeCell ref="D44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improve 表外数据录入 UX: add ★ 必填 / ⚡ 自动算 标记, clarify engine auto-fallback logic in 说明 column
</commit_message>
<xml_diff>
--- a/examples/表外数据收集表.xlsx
+++ b/examples/表外数据收集表.xlsx
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>支付给职工的工资</t>
+          <t>★ 支付给职工的工资</t>
         </is>
       </c>
       <c r="C6" s="13" t="n"/>
@@ -707,7 +707,7 @@
       <c r="F6" s="10" t="n"/>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>全年实发工资总额（含奖金津贴）★必填，直接影响经营净额</t>
+          <t>全年实发工资总额。系统不自动推算，必须手填（直接影响经营净额）</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>社保+公积金等（不填则按工资×26.6%自动推算）</t>
+          <t>社保+公积金等。留空时系统按工资×26.6%自动推算</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       <c r="F8" s="10" t="n"/>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>其他职工福利（不填则按工资×1.06%自动推算）</t>
+          <t>其他职工福利。留空时系统按工资×1.06%自动推算</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       <c r="A9" s="14" t="n"/>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>合计</t>
+          <t>⚡ 合计（工资+四金+福利费）</t>
         </is>
       </c>
       <c r="C9" s="16">
@@ -790,7 +790,7 @@
       <c r="F10" s="10" t="n"/>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>全年销项税额（不填则按收入×6%推算，请按实际税率改）</t>
+          <t>全年销项税额。留空时系统按收入×6%推算（税率默认6%，须按实际改）</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       <c r="F11" s="10" t="n"/>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>全年进项税额（不填则按成本×6%推算）</t>
+          <t>全年进项税额。留空时系统按成本×6%推算</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       <c r="A12" s="14" t="n"/>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>应交增值税</t>
+          <t>⚡ 应交增值税</t>
         </is>
       </c>
       <c r="C12" s="16">
@@ -854,7 +854,7 @@
       <c r="F13" s="10" t="n"/>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>除增值税外各税种（不填取利润表营业税金及附加）</t>
+          <t>除增值税外各税种（城建税/教育附加等）。留空时系统取利润表营业税金及附加</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       <c r="F14" s="10" t="n"/>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>全年所得税（不填取利润表所得税费用）</t>
+          <t>全年所得税。留空时系统取利润表所得税费用</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       <c r="F15" s="10" t="n"/>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>计入管理费用的税金（如房产税、印花税）</t>
+          <t>计入管理费用的税金（房产税、印花税、车船税等）</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       <c r="A17" s="14" t="n"/>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>实际应缴纳各项税金合计</t>
+          <t>⚡ 实际应缴纳各项税金合计</t>
         </is>
       </c>
       <c r="C17" s="16">
@@ -994,7 +994,7 @@
       <c r="F20" s="10" t="n"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>利息支出总额（不抵减利息收入；即利润表财务费用中的利息部分）</t>
+          <t>利息支出（不抵减利息收入；利润表财务费用中的利息部分）</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       <c r="A21" s="14" t="n"/>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>分配股利、利润或偿付利息所支付的现金</t>
+          <t>⚡ 分配股利、利润或偿付利息所支付的现金</t>
         </is>
       </c>
       <c r="C21" s="16">
@@ -1603,62 +1603,54 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="24" t="inlineStr">
         <is>
-          <t>※ ★ 必填项只有：支付给职工的工资。其余均可留空由引擎自动推算/置0。</t>
+          <t>※ ★ = 必填项（系统不自动推算，必须手填）。⚡ = 自动算公式（粉红阴影，不要填）。其他 = 选填（留空时系统按说明自动推算）。</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="24" t="inlineStr">
         <is>
-          <t>※ ★ 金额单位：元。直接填数字，不要带千分位逗号。</t>
+          <t>※ ★ 全年实发工资是唯一必填项；其余留空时系统自动按默认比例推算（详见每个项目的「说明」列）。</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="24" t="inlineStr">
         <is>
-          <t>※ ★ 粉红阴影 = 公式自动算，不要手填（手填会让 Excel 报错）。</t>
+          <t>※ ★ 税率列默认值：销项 6% / 进项 0% / 所得税 25% / 坏账 0.5%，请按公司实际修改。</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="24" t="inlineStr">
         <is>
-          <t>※ ★ 税率列默认值与原模板一致（销项 6% / 进项 0% / 所得税 25% / 坏账 0.5%），请按公司实际修改。</t>
+          <t>※ ★ 数据来源列（浅蓝）：建议每个数字注明出处（如「管理费用明细-工资」），便于审计追溯。</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="24" t="inlineStr">
         <is>
-          <t>※ ★ 数据来源列（浅蓝）：建议每填一个数字就在这列注明出处（如'管理费用明细-工资'、'税务申报表-增值税'），便于审计追溯。</t>
+          <t>※ ★ 填完后保存，运行时作为 --extra 参数传入：python cash_flow_generator.py --bs 资产负债表 --pl 利润表 --extra 表外数据收集表.xlsx</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="24" t="inlineStr">
         <is>
-          <t>※ ★ 填完后保存，运行时作为 --extra 参数传入：python cash_flow_generator.py --bs 资产负债表 --pl 利润表 --extra 表外数据收集表.xlsx</t>
+          <t>※ ★ 补齐本表后，「经营活动产生的现金流量净额」精度可由 ±20% 提升至 ±5% 以内。</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="24" t="inlineStr">
         <is>
-          <t>※ ★ 补齐本表后，'经营活动产生的现金流量净额'精度可由 ±20% 提升至 ±5% 以内。</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="24" t="inlineStr">
-        <is>
           <t>※ ★ 数据来源建议：工资表/社保申报表、增值税及所得税申报表、固定资产折旧明细表、银行对账单。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="A62:G62"/>
+  <mergeCells count="23">
     <mergeCell ref="D46:E46"/>
     <mergeCell ref="D50:E50"/>
     <mergeCell ref="D45:E45"/>

</xml_diff>